<commit_message>
add density maps more clear, combine eh&b sheets into 1
</commit_message>
<xml_diff>
--- a/Decisions/EH&B/State Region Density Maps.xlsx
+++ b/Decisions/EH&B/State Region Density Maps.xlsx
@@ -790,7 +790,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Charter leads on residential locations in 19 states vs Comcast in 27 (5 neither); the location margin is +5.54M units in New York and -4.36M in Pennsylvania, and by Census division Charter’s only positive unit-margin clusters are East North Central (-0.41M, 2 lead states) and West South Central (+3.55M, Texas-driven) while South Atlantic is -3.57M and Middle Atlantic -1.12M.</t>
+          <t>Charter leads Comcast on residential locations in 19 of 51 states (+5.54M units in New York) against 27 Comcast-lead states (-4.36M in Pennsylvania); by Census division the only positive Charter unit margins are West South Central (+3.55M, Texas-driven), West North Central (+1.19M), and East South Central (+0.44M).</t>
         </is>
       </c>
     </row>
@@ -6965,7 +6965,7 @@
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Charter leads on residential locations in 19 states vs Comcast in 27 (5 neither); the location margin is +5.54M units in New York and -4.36M in Pennsylvania, and by Census division Charter’s only positive unit-margin clusters are East North Central (-0.41M, 2 lead states) and West South Central (+3.55M, Texas-driven) while South Atlantic is -3.57M and Middle Atlantic -1.12M.</t>
+          <t>Charter leads Comcast on residential locations in 19 of 51 states (+5.54M units in New York) against 27 Comcast-lead states (-4.36M in Pennsylvania); by Census division the only positive Charter unit margins are West South Central (+3.55M, Texas-driven), West North Central (+1.19M), and East South Central (+0.44M).</t>
         </is>
       </c>
     </row>

</xml_diff>